<commit_message>
Actualización SNIES y dashboard: 2026-09-15
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V190"/>
+  <dimension ref="A1:V191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -18878,10 +18878,8 @@
       </c>
     </row>
     <row r="189">
-      <c r="A189" t="inlineStr">
-        <is>
-          <t>1720</t>
-        </is>
+      <c r="A189" t="n">
+        <v>1720</v>
       </c>
       <c r="B189" t="inlineStr">
         <is>
@@ -18933,7 +18931,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N189" s="2" t="n">
+      <c r="N189" s="1" t="n">
         <v>43816</v>
       </c>
       <c r="O189" t="inlineStr">
@@ -18974,10 +18972,8 @@
       </c>
     </row>
     <row r="190">
-      <c r="A190" t="inlineStr">
-        <is>
-          <t>3713</t>
-        </is>
+      <c r="A190" t="n">
+        <v>3713</v>
       </c>
       <c r="B190" t="inlineStr">
         <is>
@@ -19031,7 +19027,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N190" s="2" t="n">
+      <c r="N190" s="1" t="n">
         <v>44384</v>
       </c>
       <c r="O190" t="inlineStr">
@@ -19066,6 +19062,104 @@
         </is>
       </c>
       <c r="V190" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
+          <t>4721</t>
+        </is>
+      </c>
+      <c r="B191" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSITARIA HORIZONTE</t>
+        </is>
+      </c>
+      <c r="C191" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D191" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F191" t="n">
+        <v>109386</v>
+      </c>
+      <c r="G191" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION AGROPECUARIA</t>
+        </is>
+      </c>
+      <c r="H191" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I191" t="n">
+        <v>148</v>
+      </c>
+      <c r="J191" t="n">
+        <v>9</v>
+      </c>
+      <c r="K191" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L191" t="n">
+        <v>6602600</v>
+      </c>
+      <c r="M191" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N191" s="2" t="n">
+        <v>44054</v>
+      </c>
+      <c r="O191" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P191" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q191" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R191" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S191" t="inlineStr"/>
+      <c r="T191" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="U191" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V191" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-09-22
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V191"/>
+  <dimension ref="A1:V194"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19068,10 +19068,8 @@
       </c>
     </row>
     <row r="191">
-      <c r="A191" t="inlineStr">
-        <is>
-          <t>4721</t>
-        </is>
+      <c r="A191" t="n">
+        <v>4721</v>
       </c>
       <c r="B191" t="inlineStr">
         <is>
@@ -19125,7 +19123,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N191" s="2" t="n">
+      <c r="N191" s="1" t="n">
         <v>44054</v>
       </c>
       <c r="O191" t="inlineStr">
@@ -19160,6 +19158,298 @@
         </is>
       </c>
       <c r="V191" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" t="inlineStr">
+        <is>
+          <t>1110</t>
+        </is>
+      </c>
+      <c r="B192" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DEL CAUCA</t>
+        </is>
+      </c>
+      <c r="C192" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="D192" t="inlineStr">
+        <is>
+          <t>Cauca</t>
+        </is>
+      </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>Popayán</t>
+        </is>
+      </c>
+      <c r="F192" t="n">
+        <v>15440</v>
+      </c>
+      <c r="G192" t="inlineStr">
+        <is>
+          <t>LICENCIATURA EN ETNOEDUCACION</t>
+        </is>
+      </c>
+      <c r="H192" t="inlineStr">
+        <is>
+          <t>A distancia</t>
+        </is>
+      </c>
+      <c r="I192" t="n">
+        <v>152</v>
+      </c>
+      <c r="J192" t="n">
+        <v>10</v>
+      </c>
+      <c r="K192" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L192" t="n">
+        <v>245789</v>
+      </c>
+      <c r="M192" t="inlineStr">
+        <is>
+          <t>Anual</t>
+        </is>
+      </c>
+      <c r="N192" s="2" t="n">
+        <v>43315</v>
+      </c>
+      <c r="O192" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="P192" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="Q192" t="inlineStr">
+        <is>
+          <t>Formación para docentes sin asignatura de especialización</t>
+        </is>
+      </c>
+      <c r="R192" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="S192" t="inlineStr"/>
+      <c r="T192" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="U192" t="inlineStr">
+        <is>
+          <t>Instituto de Estudios en Educación</t>
+        </is>
+      </c>
+      <c r="V192" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" t="inlineStr">
+        <is>
+          <t>1710</t>
+        </is>
+      </c>
+      <c r="B193" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD PONTIFICIA BOLIVARIANA</t>
+        </is>
+      </c>
+      <c r="C193" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D193" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F193" t="n">
+        <v>119356</v>
+      </c>
+      <c r="G193" t="inlineStr">
+        <is>
+          <t>INGENIERÍA EN INTELIGENCIA ARTIFICIAL Y CIENCIA DE DATOS</t>
+        </is>
+      </c>
+      <c r="H193" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="I193" t="n">
+        <v>133</v>
+      </c>
+      <c r="J193" t="n">
+        <v>8</v>
+      </c>
+      <c r="K193" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L193" t="inlineStr"/>
+      <c r="M193" t="inlineStr">
+        <is>
+          <t>Bimensual</t>
+        </is>
+      </c>
+      <c r="N193" s="2" t="n">
+        <v>46154</v>
+      </c>
+      <c r="O193" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="P193" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="Q193" t="inlineStr">
+        <is>
+          <t>Desarrollo y análisis de software y aplicaciones</t>
+        </is>
+      </c>
+      <c r="R193" t="inlineStr">
+        <is>
+          <t>Ingeniería de sistemas, telemática y afines</t>
+        </is>
+      </c>
+      <c r="S193" t="inlineStr"/>
+      <c r="T193" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="U193" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V193" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" t="inlineStr">
+        <is>
+          <t>1828</t>
+        </is>
+      </c>
+      <c r="B194" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD ICESI</t>
+        </is>
+      </c>
+      <c r="C194" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D194" t="inlineStr">
+        <is>
+          <t>Valle del Cauca</t>
+        </is>
+      </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>Santiago de Cali</t>
+        </is>
+      </c>
+      <c r="F194" t="n">
+        <v>5093</v>
+      </c>
+      <c r="G194" t="inlineStr">
+        <is>
+          <t>INGENIERIA TELEMATICA</t>
+        </is>
+      </c>
+      <c r="H194" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I194" t="n">
+        <v>167</v>
+      </c>
+      <c r="J194" t="n">
+        <v>10</v>
+      </c>
+      <c r="K194" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L194" t="n">
+        <v>14879556</v>
+      </c>
+      <c r="M194" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N194" s="2" t="n">
+        <v>43144</v>
+      </c>
+      <c r="O194" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="P194" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="Q194" t="inlineStr">
+        <is>
+          <t>Diseño y administración de redes y bases de datos</t>
+        </is>
+      </c>
+      <c r="R194" t="inlineStr">
+        <is>
+          <t>Ingeniería de sistemas, telemática y afines</t>
+        </is>
+      </c>
+      <c r="S194" t="inlineStr"/>
+      <c r="T194" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="U194" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V194" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-09-29
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V194"/>
+  <dimension ref="A1:V200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19164,10 +19164,8 @@
       </c>
     </row>
     <row r="192">
-      <c r="A192" t="inlineStr">
-        <is>
-          <t>1110</t>
-        </is>
+      <c r="A192" t="n">
+        <v>1110</v>
       </c>
       <c r="B192" t="inlineStr">
         <is>
@@ -19221,7 +19219,7 @@
           <t>Anual</t>
         </is>
       </c>
-      <c r="N192" s="2" t="n">
+      <c r="N192" s="1" t="n">
         <v>43315</v>
       </c>
       <c r="O192" t="inlineStr">
@@ -19262,10 +19260,8 @@
       </c>
     </row>
     <row r="193">
-      <c r="A193" t="inlineStr">
-        <is>
-          <t>1710</t>
-        </is>
+      <c r="A193" t="n">
+        <v>1710</v>
       </c>
       <c r="B193" t="inlineStr">
         <is>
@@ -19317,7 +19313,7 @@
           <t>Bimensual</t>
         </is>
       </c>
-      <c r="N193" s="2" t="n">
+      <c r="N193" s="1" t="n">
         <v>46154</v>
       </c>
       <c r="O193" t="inlineStr">
@@ -19358,10 +19354,8 @@
       </c>
     </row>
     <row r="194">
-      <c r="A194" t="inlineStr">
-        <is>
-          <t>1828</t>
-        </is>
+      <c r="A194" t="n">
+        <v>1828</v>
       </c>
       <c r="B194" t="inlineStr">
         <is>
@@ -19415,7 +19409,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N194" s="2" t="n">
+      <c r="N194" s="1" t="n">
         <v>43144</v>
       </c>
       <c r="O194" t="inlineStr">
@@ -19450,6 +19444,586 @@
         </is>
       </c>
       <c r="V194" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" t="inlineStr">
+        <is>
+          <t>1207</t>
+        </is>
+      </c>
+      <c r="B195" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DEL TOLIMA</t>
+        </is>
+      </c>
+      <c r="C195" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="D195" t="inlineStr">
+        <is>
+          <t>Tolima</t>
+        </is>
+      </c>
+      <c r="E195" t="inlineStr">
+        <is>
+          <t>Ibagué</t>
+        </is>
+      </c>
+      <c r="F195" t="n">
+        <v>119127</v>
+      </c>
+      <c r="G195" t="inlineStr">
+        <is>
+          <t>Especialización en Evaluación y Gestión de Políticas Públicas para la Igualdad Social</t>
+        </is>
+      </c>
+      <c r="H195" t="inlineStr">
+        <is>
+          <t>A distancia</t>
+        </is>
+      </c>
+      <c r="I195" t="n">
+        <v>23</v>
+      </c>
+      <c r="J195" t="n">
+        <v>2</v>
+      </c>
+      <c r="K195" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L195" t="inlineStr"/>
+      <c r="M195" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N195" s="2" t="n">
+        <v>46148</v>
+      </c>
+      <c r="O195" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P195" t="inlineStr">
+        <is>
+          <t>Ciencias sociales y del comportamiento</t>
+        </is>
+      </c>
+      <c r="Q195" t="inlineStr">
+        <is>
+          <t>Ciencias políticas y educación cívica</t>
+        </is>
+      </c>
+      <c r="R195" t="inlineStr">
+        <is>
+          <t>Ciencia política, relaciones internacionales</t>
+        </is>
+      </c>
+      <c r="S195" t="inlineStr"/>
+      <c r="T195" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U195" t="inlineStr">
+        <is>
+          <t>Derecho, C. Política y Rel. Internacionales</t>
+        </is>
+      </c>
+      <c r="V195" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" t="inlineStr">
+        <is>
+          <t>1707</t>
+        </is>
+      </c>
+      <c r="B196" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE BOGOTA - JORGE TADEO LOZANO</t>
+        </is>
+      </c>
+      <c r="C196" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D196" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="E196" t="inlineStr">
+        <is>
+          <t>Cartagena de Indias</t>
+        </is>
+      </c>
+      <c r="F196" t="n">
+        <v>104914</v>
+      </c>
+      <c r="G196" t="inlineStr">
+        <is>
+          <t>COMERCIO INTERNACIONAL Y FINANZAS</t>
+        </is>
+      </c>
+      <c r="H196" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I196" t="n">
+        <v>130</v>
+      </c>
+      <c r="J196" t="n">
+        <v>8</v>
+      </c>
+      <c r="K196" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L196" t="inlineStr"/>
+      <c r="M196" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N196" s="2" t="n">
+        <v>42262</v>
+      </c>
+      <c r="O196" t="inlineStr">
+        <is>
+          <t>Ciencias Sociales, Periodismo e Información</t>
+        </is>
+      </c>
+      <c r="P196" t="inlineStr">
+        <is>
+          <t>Ciencias sociales y del comportamiento</t>
+        </is>
+      </c>
+      <c r="Q196" t="inlineStr">
+        <is>
+          <t>Economía</t>
+        </is>
+      </c>
+      <c r="R196" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S196" t="inlineStr"/>
+      <c r="T196" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U196" t="inlineStr">
+        <is>
+          <t>Humanidades y Cs. Sociales</t>
+        </is>
+      </c>
+      <c r="V196" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="197">
+      <c r="A197" t="inlineStr">
+        <is>
+          <t>1707</t>
+        </is>
+      </c>
+      <c r="B197" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE BOGOTA - JORGE TADEO LOZANO</t>
+        </is>
+      </c>
+      <c r="C197" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D197" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="E197" t="inlineStr">
+        <is>
+          <t>Cartagena de Indias</t>
+        </is>
+      </c>
+      <c r="F197" t="n">
+        <v>108043</v>
+      </c>
+      <c r="G197" t="inlineStr">
+        <is>
+          <t>MERCADEO Y PUBLICIDAD</t>
+        </is>
+      </c>
+      <c r="H197" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I197" t="n">
+        <v>134</v>
+      </c>
+      <c r="J197" t="n">
+        <v>8</v>
+      </c>
+      <c r="K197" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L197" t="inlineStr"/>
+      <c r="M197" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N197" s="2" t="n">
+        <v>43609</v>
+      </c>
+      <c r="O197" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P197" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q197" t="inlineStr">
+        <is>
+          <t>Mercadotecnia y publicidad</t>
+        </is>
+      </c>
+      <c r="R197" t="inlineStr">
+        <is>
+          <t>Publicidad y afines</t>
+        </is>
+      </c>
+      <c r="S197" t="inlineStr"/>
+      <c r="T197" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U197" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V197" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="198">
+      <c r="A198" t="inlineStr">
+        <is>
+          <t>1707</t>
+        </is>
+      </c>
+      <c r="B198" t="inlineStr">
+        <is>
+          <t>FUNDACION UNIVERSIDAD DE BOGOTA - JORGE TADEO LOZANO</t>
+        </is>
+      </c>
+      <c r="C198" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D198" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="E198" t="inlineStr">
+        <is>
+          <t>Cartagena de Indias</t>
+        </is>
+      </c>
+      <c r="F198" t="n">
+        <v>108010</v>
+      </c>
+      <c r="G198" t="inlineStr">
+        <is>
+          <t>NEGOCIOS INTERNACIONALES Y MERCADEO</t>
+        </is>
+      </c>
+      <c r="H198" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I198" t="n">
+        <v>134</v>
+      </c>
+      <c r="J198" t="n">
+        <v>8</v>
+      </c>
+      <c r="K198" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L198" t="inlineStr"/>
+      <c r="M198" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N198" s="2" t="n">
+        <v>43592</v>
+      </c>
+      <c r="O198" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P198" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q198" t="inlineStr">
+        <is>
+          <t>Mercadotecnia y publicidad</t>
+        </is>
+      </c>
+      <c r="R198" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S198" t="inlineStr"/>
+      <c r="T198" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U198" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V198" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="199">
+      <c r="A199" t="inlineStr">
+        <is>
+          <t>2747</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>INSTITUCIÓN UNIVERSITARIA VISIÓN DE LAS AMÉRICAS</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D199" t="inlineStr">
+        <is>
+          <t>Risaralda</t>
+        </is>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>Pereira</t>
+        </is>
+      </c>
+      <c r="F199" t="n">
+        <v>105923</v>
+      </c>
+      <c r="G199" t="inlineStr">
+        <is>
+          <t>MEDICINA VETERINARIA Y ZOOTECNIA</t>
+        </is>
+      </c>
+      <c r="H199" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I199" t="n">
+        <v>191</v>
+      </c>
+      <c r="J199" t="n">
+        <v>10</v>
+      </c>
+      <c r="K199" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L199" t="n">
+        <v>13235816</v>
+      </c>
+      <c r="M199" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N199" s="2" t="n">
+        <v>42670</v>
+      </c>
+      <c r="O199" t="inlineStr">
+        <is>
+          <t>Agropecuario, Silvicultura, Pesca y Veterinaria</t>
+        </is>
+      </c>
+      <c r="P199" t="inlineStr">
+        <is>
+          <t>Veterinaria</t>
+        </is>
+      </c>
+      <c r="Q199" t="inlineStr">
+        <is>
+          <t>Veterinaria</t>
+        </is>
+      </c>
+      <c r="R199" t="inlineStr">
+        <is>
+          <t>Medicina veterinaria</t>
+        </is>
+      </c>
+      <c r="S199" t="inlineStr"/>
+      <c r="T199" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U199" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="V199" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
+          <t>2747</t>
+        </is>
+      </c>
+      <c r="B200" t="inlineStr">
+        <is>
+          <t>INSTITUCIÓN UNIVERSITARIA VISIÓN DE LAS AMÉRICAS</t>
+        </is>
+      </c>
+      <c r="C200" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D200" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F200" t="n">
+        <v>53907</v>
+      </c>
+      <c r="G200" t="inlineStr">
+        <is>
+          <t>MEDICINA VETERINARIA Y ZOOTECNIA</t>
+        </is>
+      </c>
+      <c r="H200" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I200" t="n">
+        <v>189</v>
+      </c>
+      <c r="J200" t="n">
+        <v>10</v>
+      </c>
+      <c r="K200" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L200" t="n">
+        <v>12446062</v>
+      </c>
+      <c r="M200" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N200" s="2" t="n">
+        <v>39686</v>
+      </c>
+      <c r="O200" t="inlineStr">
+        <is>
+          <t>Agropecuario, Silvicultura, Pesca y Veterinaria</t>
+        </is>
+      </c>
+      <c r="P200" t="inlineStr">
+        <is>
+          <t>Veterinaria</t>
+        </is>
+      </c>
+      <c r="Q200" t="inlineStr">
+        <is>
+          <t>Veterinaria</t>
+        </is>
+      </c>
+      <c r="R200" t="inlineStr">
+        <is>
+          <t>Medicina veterinaria</t>
+        </is>
+      </c>
+      <c r="S200" t="inlineStr"/>
+      <c r="T200" t="inlineStr">
+        <is>
+          <t>2026-09-29</t>
+        </is>
+      </c>
+      <c r="U200" t="inlineStr">
+        <is>
+          <t>Otro</t>
+        </is>
+      </c>
+      <c r="V200" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-10-06
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V200"/>
+  <dimension ref="A1:V202"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -19450,10 +19450,8 @@
       </c>
     </row>
     <row r="195">
-      <c r="A195" t="inlineStr">
-        <is>
-          <t>1207</t>
-        </is>
+      <c r="A195" t="n">
+        <v>1207</v>
       </c>
       <c r="B195" t="inlineStr">
         <is>
@@ -19505,7 +19503,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N195" s="2" t="n">
+      <c r="N195" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="O195" t="inlineStr">
@@ -19546,10 +19544,8 @@
       </c>
     </row>
     <row r="196">
-      <c r="A196" t="inlineStr">
-        <is>
-          <t>1707</t>
-        </is>
+      <c r="A196" t="n">
+        <v>1707</v>
       </c>
       <c r="B196" t="inlineStr">
         <is>
@@ -19601,7 +19597,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N196" s="2" t="n">
+      <c r="N196" s="1" t="n">
         <v>42262</v>
       </c>
       <c r="O196" t="inlineStr">
@@ -19642,10 +19638,8 @@
       </c>
     </row>
     <row r="197">
-      <c r="A197" t="inlineStr">
-        <is>
-          <t>1707</t>
-        </is>
+      <c r="A197" t="n">
+        <v>1707</v>
       </c>
       <c r="B197" t="inlineStr">
         <is>
@@ -19697,7 +19691,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N197" s="2" t="n">
+      <c r="N197" s="1" t="n">
         <v>43609</v>
       </c>
       <c r="O197" t="inlineStr">
@@ -19738,10 +19732,8 @@
       </c>
     </row>
     <row r="198">
-      <c r="A198" t="inlineStr">
-        <is>
-          <t>1707</t>
-        </is>
+      <c r="A198" t="n">
+        <v>1707</v>
       </c>
       <c r="B198" t="inlineStr">
         <is>
@@ -19793,7 +19785,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N198" s="2" t="n">
+      <c r="N198" s="1" t="n">
         <v>43592</v>
       </c>
       <c r="O198" t="inlineStr">
@@ -19834,10 +19826,8 @@
       </c>
     </row>
     <row r="199">
-      <c r="A199" t="inlineStr">
-        <is>
-          <t>2747</t>
-        </is>
+      <c r="A199" t="n">
+        <v>2747</v>
       </c>
       <c r="B199" t="inlineStr">
         <is>
@@ -19891,7 +19881,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N199" s="2" t="n">
+      <c r="N199" s="1" t="n">
         <v>42670</v>
       </c>
       <c r="O199" t="inlineStr">
@@ -19932,10 +19922,8 @@
       </c>
     </row>
     <row r="200">
-      <c r="A200" t="inlineStr">
-        <is>
-          <t>2747</t>
-        </is>
+      <c r="A200" t="n">
+        <v>2747</v>
       </c>
       <c r="B200" t="inlineStr">
         <is>
@@ -19989,7 +19977,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N200" s="2" t="n">
+      <c r="N200" s="1" t="n">
         <v>39686</v>
       </c>
       <c r="O200" t="inlineStr">
@@ -20024,6 +20012,200 @@
         </is>
       </c>
       <c r="V200" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" t="inlineStr">
+        <is>
+          <t>2825</t>
+        </is>
+      </c>
+      <c r="B201" t="inlineStr">
+        <is>
+          <t>CORPORACION UNIVERSITARIA RAFAEL NUÑEZ</t>
+        </is>
+      </c>
+      <c r="C201" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D201" t="inlineStr">
+        <is>
+          <t>Bolívar</t>
+        </is>
+      </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>Cartagena de Indias</t>
+        </is>
+      </c>
+      <c r="F201" t="n">
+        <v>4448</v>
+      </c>
+      <c r="G201" t="inlineStr">
+        <is>
+          <t>BACTERIOLOGIA</t>
+        </is>
+      </c>
+      <c r="H201" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I201" t="n">
+        <v>164</v>
+      </c>
+      <c r="J201" t="n">
+        <v>10</v>
+      </c>
+      <c r="K201" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L201" t="n">
+        <v>6488640</v>
+      </c>
+      <c r="M201" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N201" s="2" t="n">
+        <v>35875</v>
+      </c>
+      <c r="O201" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P201" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q201" t="inlineStr">
+        <is>
+          <t>Tecnología de diagnóstico y tratamiento médico</t>
+        </is>
+      </c>
+      <c r="R201" t="inlineStr">
+        <is>
+          <t>Bacteriología</t>
+        </is>
+      </c>
+      <c r="S201" t="inlineStr"/>
+      <c r="T201" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="U201" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="V201" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" t="inlineStr">
+        <is>
+          <t>3204</t>
+        </is>
+      </c>
+      <c r="B202" t="inlineStr">
+        <is>
+          <t>TECNOLOGICO DE ANTIOQUIA</t>
+        </is>
+      </c>
+      <c r="C202" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="D202" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E202" t="inlineStr">
+        <is>
+          <t>Copacabana</t>
+        </is>
+      </c>
+      <c r="F202" t="n">
+        <v>102925</v>
+      </c>
+      <c r="G202" t="inlineStr">
+        <is>
+          <t>LICENCIATURA EN EDUCACIÓN PREESCOLAR</t>
+        </is>
+      </c>
+      <c r="H202" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I202" t="n">
+        <v>168</v>
+      </c>
+      <c r="J202" t="n">
+        <v>10</v>
+      </c>
+      <c r="K202" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L202" t="inlineStr"/>
+      <c r="M202" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N202" s="2" t="n">
+        <v>41610</v>
+      </c>
+      <c r="O202" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="P202" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="Q202" t="inlineStr">
+        <is>
+          <t>Formación para docentes sin asignatura de especialización</t>
+        </is>
+      </c>
+      <c r="R202" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="S202" t="inlineStr"/>
+      <c r="T202" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="U202" t="inlineStr">
+        <is>
+          <t>Instituto de Estudios en Educación</t>
+        </is>
+      </c>
+      <c r="V202" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-10-13
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V202"/>
+  <dimension ref="A1:V203"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20018,10 +20018,8 @@
       </c>
     </row>
     <row r="201">
-      <c r="A201" t="inlineStr">
-        <is>
-          <t>2825</t>
-        </is>
+      <c r="A201" t="n">
+        <v>2825</v>
       </c>
       <c r="B201" t="inlineStr">
         <is>
@@ -20075,7 +20073,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N201" s="2" t="n">
+      <c r="N201" s="1" t="n">
         <v>35875</v>
       </c>
       <c r="O201" t="inlineStr">
@@ -20116,10 +20114,8 @@
       </c>
     </row>
     <row r="202">
-      <c r="A202" t="inlineStr">
-        <is>
-          <t>3204</t>
-        </is>
+      <c r="A202" t="n">
+        <v>3204</v>
       </c>
       <c r="B202" t="inlineStr">
         <is>
@@ -20171,7 +20167,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N202" s="2" t="n">
+      <c r="N202" s="1" t="n">
         <v>41610</v>
       </c>
       <c r="O202" t="inlineStr">
@@ -20206,6 +20202,104 @@
         </is>
       </c>
       <c r="V202" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" t="inlineStr">
+        <is>
+          <t>2829</t>
+        </is>
+      </c>
+      <c r="B203" t="inlineStr">
+        <is>
+          <t>CORPORACION UNIVERSITARIA MINUTO DE DIOS -UNIMINUTO-</t>
+        </is>
+      </c>
+      <c r="C203" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D203" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F203" t="n">
+        <v>106862</v>
+      </c>
+      <c r="G203" t="inlineStr">
+        <is>
+          <t>Licenciatura en Lenguas Extranjeras con Énfasis en Inglés</t>
+        </is>
+      </c>
+      <c r="H203" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I203" t="n">
+        <v>160</v>
+      </c>
+      <c r="J203" t="n">
+        <v>10</v>
+      </c>
+      <c r="K203" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L203" t="n">
+        <v>4013700</v>
+      </c>
+      <c r="M203" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N203" s="2" t="n">
+        <v>43670</v>
+      </c>
+      <c r="O203" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="P203" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="Q203" t="inlineStr">
+        <is>
+          <t>Ciencias de la educación</t>
+        </is>
+      </c>
+      <c r="R203" t="inlineStr">
+        <is>
+          <t>Educación</t>
+        </is>
+      </c>
+      <c r="S203" t="inlineStr"/>
+      <c r="T203" t="inlineStr">
+        <is>
+          <t>2026-10-13</t>
+        </is>
+      </c>
+      <c r="U203" t="inlineStr">
+        <is>
+          <t>Instituto de Estudios en Educación</t>
+        </is>
+      </c>
+      <c r="V203" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-10-20
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V203"/>
+  <dimension ref="A1:V218"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -20208,10 +20208,8 @@
       </c>
     </row>
     <row r="203">
-      <c r="A203" t="inlineStr">
-        <is>
-          <t>2829</t>
-        </is>
+      <c r="A203" t="n">
+        <v>2829</v>
       </c>
       <c r="B203" t="inlineStr">
         <is>
@@ -20265,7 +20263,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N203" s="2" t="n">
+      <c r="N203" s="1" t="n">
         <v>43670</v>
       </c>
       <c r="O203" t="inlineStr">
@@ -20300,6 +20298,1464 @@
         </is>
       </c>
       <c r="V203" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" t="inlineStr">
+        <is>
+          <t>1833</t>
+        </is>
+      </c>
+      <c r="B204" t="inlineStr">
+        <is>
+          <t>CORPORACIÓN UNIVERSIDAD DEL SINU - ELIAS BECHARA ZAINUM - UNISINU -</t>
+        </is>
+      </c>
+      <c r="C204" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D204" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F204" t="n">
+        <v>102869</v>
+      </c>
+      <c r="G204" t="inlineStr">
+        <is>
+          <t>ADMINISTRACIÓN DE EMPRESAS</t>
+        </is>
+      </c>
+      <c r="H204" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I204" t="n">
+        <v>140</v>
+      </c>
+      <c r="J204" t="n">
+        <v>8</v>
+      </c>
+      <c r="K204" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L204" t="inlineStr"/>
+      <c r="M204" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N204" s="2" t="n">
+        <v>41599</v>
+      </c>
+      <c r="O204" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P204" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q204" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R204" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S204" t="inlineStr"/>
+      <c r="T204" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U204" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V204" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="205">
+      <c r="A205" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B205" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C205" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D205" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F205" t="n">
+        <v>6632</v>
+      </c>
+      <c r="G205" t="inlineStr">
+        <is>
+          <t>ADMINISTRACION DE NEGOCIOS INTERNACIONALES</t>
+        </is>
+      </c>
+      <c r="H205" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I205" t="n">
+        <v>168</v>
+      </c>
+      <c r="J205" t="n">
+        <v>10</v>
+      </c>
+      <c r="K205" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L205" t="n">
+        <v>5617000</v>
+      </c>
+      <c r="M205" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N205" s="2" t="n">
+        <v>35963</v>
+      </c>
+      <c r="O205" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P205" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q205" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R205" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S205" t="inlineStr"/>
+      <c r="T205" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U205" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V205" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="206">
+      <c r="A206" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B206" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C206" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D206" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E206" t="inlineStr">
+        <is>
+          <t>San José de Cúcuta</t>
+        </is>
+      </c>
+      <c r="F206" t="n">
+        <v>52353</v>
+      </c>
+      <c r="G206" t="inlineStr">
+        <is>
+          <t>ENFERMERIA</t>
+        </is>
+      </c>
+      <c r="H206" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I206" t="n">
+        <v>185</v>
+      </c>
+      <c r="J206" t="n">
+        <v>10</v>
+      </c>
+      <c r="K206" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L206" t="inlineStr"/>
+      <c r="M206" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N206" s="2" t="n">
+        <v>38972</v>
+      </c>
+      <c r="O206" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P206" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q206" t="inlineStr">
+        <is>
+          <t>Medicina</t>
+        </is>
+      </c>
+      <c r="R206" t="inlineStr">
+        <is>
+          <t>Enfermería</t>
+        </is>
+      </c>
+      <c r="S206" t="inlineStr"/>
+      <c r="T206" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U206" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="V206" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="207">
+      <c r="A207" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B207" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C207" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D207" t="inlineStr">
+        <is>
+          <t>Norte de Santander</t>
+        </is>
+      </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>San José de Cúcuta</t>
+        </is>
+      </c>
+      <c r="F207" t="n">
+        <v>5381</v>
+      </c>
+      <c r="G207" t="inlineStr">
+        <is>
+          <t>FISIOTERAPIA</t>
+        </is>
+      </c>
+      <c r="H207" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I207" t="n">
+        <v>174</v>
+      </c>
+      <c r="J207" t="n">
+        <v>10</v>
+      </c>
+      <c r="K207" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L207" t="inlineStr"/>
+      <c r="M207" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N207" s="2" t="n">
+        <v>35875</v>
+      </c>
+      <c r="O207" t="inlineStr">
+        <is>
+          <t>Salud y Bienestar</t>
+        </is>
+      </c>
+      <c r="P207" t="inlineStr">
+        <is>
+          <t>Salud</t>
+        </is>
+      </c>
+      <c r="Q207" t="inlineStr">
+        <is>
+          <t>Fisioterapia, Fonoaudiología, Terapia ocupacional, Nutrición y afines</t>
+        </is>
+      </c>
+      <c r="R207" t="inlineStr">
+        <is>
+          <t>Terapias</t>
+        </is>
+      </c>
+      <c r="S207" t="inlineStr"/>
+      <c r="T207" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U207" t="inlineStr">
+        <is>
+          <t>Ciencias de la Salud</t>
+        </is>
+      </c>
+      <c r="V207" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="208">
+      <c r="A208" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B208" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C208" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D208" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="E208" t="inlineStr">
+        <is>
+          <t>Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F208" t="n">
+        <v>102898</v>
+      </c>
+      <c r="G208" t="inlineStr">
+        <is>
+          <t>INGENIERIA AGROINDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="H208" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I208" t="n">
+        <v>170</v>
+      </c>
+      <c r="J208" t="n">
+        <v>10</v>
+      </c>
+      <c r="K208" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L208" t="inlineStr"/>
+      <c r="M208" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N208" s="2" t="n">
+        <v>41605</v>
+      </c>
+      <c r="O208" t="inlineStr">
+        <is>
+          <t>Ingeniería, Industria y Construcción</t>
+        </is>
+      </c>
+      <c r="P208" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines</t>
+        </is>
+      </c>
+      <c r="Q208" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines no clasificadas en otra parte</t>
+        </is>
+      </c>
+      <c r="R208" t="inlineStr">
+        <is>
+          <t>Ingeniería agroindustrial, alimentos y afines</t>
+        </is>
+      </c>
+      <c r="S208" t="inlineStr"/>
+      <c r="T208" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U208" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V208" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="209">
+      <c r="A209" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B209" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C209" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D209" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="E209" t="inlineStr">
+        <is>
+          <t>Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F209" t="n">
+        <v>102771</v>
+      </c>
+      <c r="G209" t="inlineStr">
+        <is>
+          <t>INGENIERÍA DE SOFTWARE</t>
+        </is>
+      </c>
+      <c r="H209" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I209" t="n">
+        <v>160</v>
+      </c>
+      <c r="J209" t="n">
+        <v>10</v>
+      </c>
+      <c r="K209" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L209" t="inlineStr"/>
+      <c r="M209" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N209" s="2" t="n">
+        <v>41522</v>
+      </c>
+      <c r="O209" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="P209" t="inlineStr">
+        <is>
+          <t>Tecnologías de la Información y la Comunicación (TIC)</t>
+        </is>
+      </c>
+      <c r="Q209" t="inlineStr">
+        <is>
+          <t>Desarrollo y análisis de software y aplicaciones</t>
+        </is>
+      </c>
+      <c r="R209" t="inlineStr">
+        <is>
+          <t>Ingeniería de sistemas, telemática y afines</t>
+        </is>
+      </c>
+      <c r="S209" t="inlineStr"/>
+      <c r="T209" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U209" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V209" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="210">
+      <c r="A210" t="inlineStr">
+        <is>
+          <t>2832</t>
+        </is>
+      </c>
+      <c r="B210" t="inlineStr">
+        <is>
+          <t>UNIVERSIDAD DE SANTANDER - UDES</t>
+        </is>
+      </c>
+      <c r="C210" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D210" t="inlineStr">
+        <is>
+          <t>Santander</t>
+        </is>
+      </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>Bucaramanga</t>
+        </is>
+      </c>
+      <c r="F210" t="n">
+        <v>105181</v>
+      </c>
+      <c r="G210" t="inlineStr">
+        <is>
+          <t>INGENIERÍA PETROQUÍMICA</t>
+        </is>
+      </c>
+      <c r="H210" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I210" t="n">
+        <v>163</v>
+      </c>
+      <c r="J210" t="n">
+        <v>10</v>
+      </c>
+      <c r="K210" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L210" t="inlineStr"/>
+      <c r="M210" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N210" s="2" t="n">
+        <v>42403</v>
+      </c>
+      <c r="O210" t="inlineStr">
+        <is>
+          <t>Ingeniería, Industria y Construcción</t>
+        </is>
+      </c>
+      <c r="P210" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines</t>
+        </is>
+      </c>
+      <c r="Q210" t="inlineStr">
+        <is>
+          <t>Ingeniería y profesiones afines no clasificadas en otra parte</t>
+        </is>
+      </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>Ingeniería de minas, metalurgia y afines</t>
+        </is>
+      </c>
+      <c r="S210" t="inlineStr"/>
+      <c r="T210" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U210" t="inlineStr">
+        <is>
+          <t>Ingenierías</t>
+        </is>
+      </c>
+      <c r="V210" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="211">
+      <c r="A211" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B211" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C211" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D211" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F211" t="n">
+        <v>102846</v>
+      </c>
+      <c r="G211" t="inlineStr">
+        <is>
+          <t>CONTADURÍA PÚBLICA</t>
+        </is>
+      </c>
+      <c r="H211" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I211" t="n">
+        <v>160</v>
+      </c>
+      <c r="J211" t="n">
+        <v>2</v>
+      </c>
+      <c r="K211" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L211" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M211" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N211" s="2" t="n">
+        <v>41573</v>
+      </c>
+      <c r="O211" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P211" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q211" t="inlineStr">
+        <is>
+          <t>Contabilidad e impuestos</t>
+        </is>
+      </c>
+      <c r="R211" t="inlineStr">
+        <is>
+          <t>Contaduría pública</t>
+        </is>
+      </c>
+      <c r="S211" t="inlineStr"/>
+      <c r="T211" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U211" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V211" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="212">
+      <c r="A212" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B212" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C212" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D212" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F212" t="n">
+        <v>105608</v>
+      </c>
+      <c r="G212" t="inlineStr">
+        <is>
+          <t>PROFESIONAL DE DISEÑO DE MODAS</t>
+        </is>
+      </c>
+      <c r="H212" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I212" t="n">
+        <v>153</v>
+      </c>
+      <c r="J212" t="n">
+        <v>2</v>
+      </c>
+      <c r="K212" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L212" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M212" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N212" s="2" t="n">
+        <v>42535</v>
+      </c>
+      <c r="O212" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P212" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q212" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R212" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="S212" t="inlineStr"/>
+      <c r="T212" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U212" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V212" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="213">
+      <c r="A213" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B213" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C213" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D213" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F213" t="n">
+        <v>102870</v>
+      </c>
+      <c r="G213" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN ADMINISTRACIÓN DE EMPRESAS</t>
+        </is>
+      </c>
+      <c r="H213" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I213" t="n">
+        <v>136</v>
+      </c>
+      <c r="J213" t="n">
+        <v>2</v>
+      </c>
+      <c r="K213" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L213" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M213" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N213" s="2" t="n">
+        <v>41599</v>
+      </c>
+      <c r="O213" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P213" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q213" t="inlineStr">
+        <is>
+          <t>Gestión y administración</t>
+        </is>
+      </c>
+      <c r="R213" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S213" t="inlineStr"/>
+      <c r="T213" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U213" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V213" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="214">
+      <c r="A214" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B214" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C214" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D214" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F214" t="n">
+        <v>106017</v>
+      </c>
+      <c r="G214" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN DISEÑO DE ESPACIOS</t>
+        </is>
+      </c>
+      <c r="H214" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I214" t="n">
+        <v>140</v>
+      </c>
+      <c r="J214" t="n">
+        <v>9</v>
+      </c>
+      <c r="K214" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L214" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M214" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N214" s="2" t="n">
+        <v>42700</v>
+      </c>
+      <c r="O214" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P214" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q214" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R214" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="S214" t="inlineStr"/>
+      <c r="T214" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U214" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V214" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="215">
+      <c r="A215" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B215" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C215" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D215" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F215" t="n">
+        <v>105779</v>
+      </c>
+      <c r="G215" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN DISEÑO INDUSTRIAL</t>
+        </is>
+      </c>
+      <c r="H215" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I215" t="n">
+        <v>156</v>
+      </c>
+      <c r="J215" t="n">
+        <v>9</v>
+      </c>
+      <c r="K215" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L215" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M215" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N215" s="2" t="n">
+        <v>42608</v>
+      </c>
+      <c r="O215" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P215" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q215" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R215" t="inlineStr">
+        <is>
+          <t>Diseño</t>
+        </is>
+      </c>
+      <c r="S215" t="inlineStr"/>
+      <c r="T215" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U215" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V215" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="216">
+      <c r="A216" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B216" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C216" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D216" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F216" t="n">
+        <v>104998</v>
+      </c>
+      <c r="G216" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN MARKETING INTERNACIONAL</t>
+        </is>
+      </c>
+      <c r="H216" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I216" t="n">
+        <v>135</v>
+      </c>
+      <c r="J216" t="n">
+        <v>2</v>
+      </c>
+      <c r="K216" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L216" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M216" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N216" s="2" t="n">
+        <v>42292</v>
+      </c>
+      <c r="O216" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P216" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q216" t="inlineStr">
+        <is>
+          <t>Mercadotecnia y publicidad</t>
+        </is>
+      </c>
+      <c r="R216" t="inlineStr">
+        <is>
+          <t>Administración</t>
+        </is>
+      </c>
+      <c r="S216" t="inlineStr"/>
+      <c r="T216" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U216" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V216" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="217">
+      <c r="A217" t="inlineStr">
+        <is>
+          <t>4702</t>
+        </is>
+      </c>
+      <c r="B217" t="inlineStr">
+        <is>
+          <t>FUNDACION DE EDUCACION SUPERIOR SAN JOSE -FESSANJOSE-</t>
+        </is>
+      </c>
+      <c r="C217" t="inlineStr">
+        <is>
+          <t>Privado</t>
+        </is>
+      </c>
+      <c r="D217" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>Bogotá, D.C.</t>
+        </is>
+      </c>
+      <c r="F217" t="n">
+        <v>105187</v>
+      </c>
+      <c r="G217" t="inlineStr">
+        <is>
+          <t>PROFESIONAL EN PUBLICIDAD</t>
+        </is>
+      </c>
+      <c r="H217" t="inlineStr">
+        <is>
+          <t>Presencial</t>
+        </is>
+      </c>
+      <c r="I217" t="n">
+        <v>145</v>
+      </c>
+      <c r="J217" t="n">
+        <v>2</v>
+      </c>
+      <c r="K217" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L217" t="n">
+        <v>4370822</v>
+      </c>
+      <c r="M217" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N217" s="2" t="n">
+        <v>42403</v>
+      </c>
+      <c r="O217" t="inlineStr">
+        <is>
+          <t>Arte y Humanidades</t>
+        </is>
+      </c>
+      <c r="P217" t="inlineStr">
+        <is>
+          <t>Artes</t>
+        </is>
+      </c>
+      <c r="Q217" t="inlineStr">
+        <is>
+          <t>Diseño industrial, de moda e interiores</t>
+        </is>
+      </c>
+      <c r="R217" t="inlineStr">
+        <is>
+          <t>Publicidad y afines</t>
+        </is>
+      </c>
+      <c r="S217" t="inlineStr"/>
+      <c r="T217" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U217" t="inlineStr">
+        <is>
+          <t>Escuela de Arquitectura, Urbanismo y Diseño</t>
+        </is>
+      </c>
+      <c r="V217" t="inlineStr">
+        <is>
+          <t>Inactivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="218">
+      <c r="A218" t="inlineStr">
+        <is>
+          <t>9927</t>
+        </is>
+      </c>
+      <c r="B218" t="inlineStr">
+        <is>
+          <t>INSTITUCION UNIVERSITARIA DIGITAL DE ANTIOQUIA -IU. DIGITAL</t>
+        </is>
+      </c>
+      <c r="C218" t="inlineStr">
+        <is>
+          <t>Oficial</t>
+        </is>
+      </c>
+      <c r="D218" t="inlineStr">
+        <is>
+          <t>Antioquia</t>
+        </is>
+      </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>Medellín</t>
+        </is>
+      </c>
+      <c r="F218" t="n">
+        <v>108269</v>
+      </c>
+      <c r="G218" t="inlineStr">
+        <is>
+          <t>PUBLICIDAD Y MERCADEO DIGITAL</t>
+        </is>
+      </c>
+      <c r="H218" t="inlineStr">
+        <is>
+          <t>Virtual</t>
+        </is>
+      </c>
+      <c r="I218" t="n">
+        <v>141</v>
+      </c>
+      <c r="J218" t="n">
+        <v>8</v>
+      </c>
+      <c r="K218" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="L218" t="n">
+        <v>2765000</v>
+      </c>
+      <c r="M218" t="inlineStr">
+        <is>
+          <t>Semestral</t>
+        </is>
+      </c>
+      <c r="N218" s="2" t="n">
+        <v>43706</v>
+      </c>
+      <c r="O218" t="inlineStr">
+        <is>
+          <t>Administración de Empresas y Derecho</t>
+        </is>
+      </c>
+      <c r="P218" t="inlineStr">
+        <is>
+          <t>Educación comercial y administración</t>
+        </is>
+      </c>
+      <c r="Q218" t="inlineStr">
+        <is>
+          <t>Mercadotecnia y publicidad</t>
+        </is>
+      </c>
+      <c r="R218" t="inlineStr">
+        <is>
+          <t>Publicidad y afines</t>
+        </is>
+      </c>
+      <c r="S218" t="inlineStr"/>
+      <c r="T218" t="inlineStr">
+        <is>
+          <t>2026-10-20</t>
+        </is>
+      </c>
+      <c r="U218" t="inlineStr">
+        <is>
+          <t>Escuela de Negocios</t>
+        </is>
+      </c>
+      <c r="V218" t="inlineStr">
         <is>
           <t>Inactivo</t>
         </is>

</xml_diff>

<commit_message>
Actualización SNIES y dashboard: 2026-10-27
</commit_message>
<xml_diff>
--- a/data/novedades/Inactivos_pregrado.xlsx
+++ b/data/novedades/Inactivos_pregrado.xlsx
@@ -16,11 +16,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
-    <numFmt numFmtId="166" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="167" formatCode="YYYY-MM-DD"/>
   </numFmts>
   <fonts count="1">
     <font>
@@ -51,10 +49,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -20304,10 +20301,8 @@
       </c>
     </row>
     <row r="204">
-      <c r="A204" t="inlineStr">
-        <is>
-          <t>1833</t>
-        </is>
+      <c r="A204" t="n">
+        <v>1833</v>
       </c>
       <c r="B204" t="inlineStr">
         <is>
@@ -20359,7 +20354,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N204" s="2" t="n">
+      <c r="N204" s="1" t="n">
         <v>41599</v>
       </c>
       <c r="O204" t="inlineStr">
@@ -20400,10 +20395,8 @@
       </c>
     </row>
     <row r="205">
-      <c r="A205" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A205" t="n">
+        <v>2832</v>
       </c>
       <c r="B205" t="inlineStr">
         <is>
@@ -20457,7 +20450,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N205" s="2" t="n">
+      <c r="N205" s="1" t="n">
         <v>35963</v>
       </c>
       <c r="O205" t="inlineStr">
@@ -20498,10 +20491,8 @@
       </c>
     </row>
     <row r="206">
-      <c r="A206" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A206" t="n">
+        <v>2832</v>
       </c>
       <c r="B206" t="inlineStr">
         <is>
@@ -20553,7 +20544,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N206" s="2" t="n">
+      <c r="N206" s="1" t="n">
         <v>38972</v>
       </c>
       <c r="O206" t="inlineStr">
@@ -20594,10 +20585,8 @@
       </c>
     </row>
     <row r="207">
-      <c r="A207" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A207" t="n">
+        <v>2832</v>
       </c>
       <c r="B207" t="inlineStr">
         <is>
@@ -20649,7 +20638,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N207" s="2" t="n">
+      <c r="N207" s="1" t="n">
         <v>35875</v>
       </c>
       <c r="O207" t="inlineStr">
@@ -20690,10 +20679,8 @@
       </c>
     </row>
     <row r="208">
-      <c r="A208" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A208" t="n">
+        <v>2832</v>
       </c>
       <c r="B208" t="inlineStr">
         <is>
@@ -20745,7 +20732,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N208" s="2" t="n">
+      <c r="N208" s="1" t="n">
         <v>41605</v>
       </c>
       <c r="O208" t="inlineStr">
@@ -20786,10 +20773,8 @@
       </c>
     </row>
     <row r="209">
-      <c r="A209" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A209" t="n">
+        <v>2832</v>
       </c>
       <c r="B209" t="inlineStr">
         <is>
@@ -20841,7 +20826,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N209" s="2" t="n">
+      <c r="N209" s="1" t="n">
         <v>41522</v>
       </c>
       <c r="O209" t="inlineStr">
@@ -20882,10 +20867,8 @@
       </c>
     </row>
     <row r="210">
-      <c r="A210" t="inlineStr">
-        <is>
-          <t>2832</t>
-        </is>
+      <c r="A210" t="n">
+        <v>2832</v>
       </c>
       <c r="B210" t="inlineStr">
         <is>
@@ -20937,7 +20920,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N210" s="2" t="n">
+      <c r="N210" s="1" t="n">
         <v>42403</v>
       </c>
       <c r="O210" t="inlineStr">
@@ -20978,10 +20961,8 @@
       </c>
     </row>
     <row r="211">
-      <c r="A211" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A211" t="n">
+        <v>4702</v>
       </c>
       <c r="B211" t="inlineStr">
         <is>
@@ -21035,7 +21016,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N211" s="2" t="n">
+      <c r="N211" s="1" t="n">
         <v>41573</v>
       </c>
       <c r="O211" t="inlineStr">
@@ -21076,10 +21057,8 @@
       </c>
     </row>
     <row r="212">
-      <c r="A212" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A212" t="n">
+        <v>4702</v>
       </c>
       <c r="B212" t="inlineStr">
         <is>
@@ -21133,7 +21112,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N212" s="2" t="n">
+      <c r="N212" s="1" t="n">
         <v>42535</v>
       </c>
       <c r="O212" t="inlineStr">
@@ -21174,10 +21153,8 @@
       </c>
     </row>
     <row r="213">
-      <c r="A213" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A213" t="n">
+        <v>4702</v>
       </c>
       <c r="B213" t="inlineStr">
         <is>
@@ -21231,7 +21208,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N213" s="2" t="n">
+      <c r="N213" s="1" t="n">
         <v>41599</v>
       </c>
       <c r="O213" t="inlineStr">
@@ -21272,10 +21249,8 @@
       </c>
     </row>
     <row r="214">
-      <c r="A214" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A214" t="n">
+        <v>4702</v>
       </c>
       <c r="B214" t="inlineStr">
         <is>
@@ -21329,7 +21304,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N214" s="2" t="n">
+      <c r="N214" s="1" t="n">
         <v>42700</v>
       </c>
       <c r="O214" t="inlineStr">
@@ -21370,10 +21345,8 @@
       </c>
     </row>
     <row r="215">
-      <c r="A215" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A215" t="n">
+        <v>4702</v>
       </c>
       <c r="B215" t="inlineStr">
         <is>
@@ -21427,7 +21400,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N215" s="2" t="n">
+      <c r="N215" s="1" t="n">
         <v>42608</v>
       </c>
       <c r="O215" t="inlineStr">
@@ -21468,10 +21441,8 @@
       </c>
     </row>
     <row r="216">
-      <c r="A216" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A216" t="n">
+        <v>4702</v>
       </c>
       <c r="B216" t="inlineStr">
         <is>
@@ -21525,7 +21496,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N216" s="2" t="n">
+      <c r="N216" s="1" t="n">
         <v>42292</v>
       </c>
       <c r="O216" t="inlineStr">
@@ -21566,10 +21537,8 @@
       </c>
     </row>
     <row r="217">
-      <c r="A217" t="inlineStr">
-        <is>
-          <t>4702</t>
-        </is>
+      <c r="A217" t="n">
+        <v>4702</v>
       </c>
       <c r="B217" t="inlineStr">
         <is>
@@ -21623,7 +21592,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N217" s="2" t="n">
+      <c r="N217" s="1" t="n">
         <v>42403</v>
       </c>
       <c r="O217" t="inlineStr">
@@ -21664,10 +21633,8 @@
       </c>
     </row>
     <row r="218">
-      <c r="A218" t="inlineStr">
-        <is>
-          <t>9927</t>
-        </is>
+      <c r="A218" t="n">
+        <v>9927</v>
       </c>
       <c r="B218" t="inlineStr">
         <is>
@@ -21721,7 +21688,7 @@
           <t>Semestral</t>
         </is>
       </c>
-      <c r="N218" s="2" t="n">
+      <c r="N218" s="1" t="n">
         <v>43706</v>
       </c>
       <c r="O218" t="inlineStr">

</xml_diff>